<commit_message>
inv list precios formato numero
</commit_message>
<xml_diff>
--- a/Macro Inv Tarde/VALORIZADO FALTANTES IMPO.xlsx
+++ b/Macro Inv Tarde/VALORIZADO FALTANTES IMPO.xlsx
@@ -397,13 +397,13 @@
     <t>Valorizado</t>
   </si>
   <si>
-    <t>Período: 30/11/2025 13:41:04</t>
+    <t>Período: 30/11/2025 13:21:00</t>
   </si>
   <si>
     <t>COLGAAP</t>
   </si>
   <si>
-    <t>Fecha y hora de generación: 05/11/2025 13:41:37</t>
+    <t>Fecha y hora de generación: 06/11/2025 13:21:33</t>
   </si>
 </sst>
 </file>

</xml_diff>